<commit_message>
Replace long dashes with hyphens across v2 deliverables
Sanitize em dash, en dash and minus sign to hyphen in all three v2
files (deck, xlsx, doc); reword '->20%' style strings to 'drops >20%'.

https://claude.ai/code/session_01NksSqrSqDgtmZbhunqjgZD
</commit_message>
<xml_diff>
--- a/outputs/touchretouch-testtask/v2/TouchRetouch_ROAS_Model.xlsx
+++ b/outputs/touchretouch-testtask/v2/TouchRetouch_ROAS_Model.xlsx
@@ -617,7 +617,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TouchRetouch — ASA Funnel &amp; ROAS Model</t>
+          <t>TouchRetouch - ASA Funnel &amp; ROAS Model</t>
         </is>
       </c>
     </row>
@@ -628,6 +628,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -736,7 +737,7 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Info only (not in gate) — pull real D30/Y1 curve from RevenueCat</t>
+          <t>Info only (not in gate) - pull real D30/Y1 curve from RevenueCat</t>
         </is>
       </c>
     </row>
@@ -760,6 +761,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
@@ -834,6 +836,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
         <is>
@@ -892,6 +895,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
         <is>
@@ -972,7 +976,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>M0 — Baseline (current)</t>
+          <t>M0 - Baseline (current)</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
@@ -1031,7 +1035,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>M1 — Bank efficiency</t>
+          <t>M1 - Bank efficiency</t>
         </is>
       </c>
       <c r="B6" s="18" t="n">
@@ -1090,7 +1094,7 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>M2 — Gate cleared</t>
+          <t>M2 - Gate cleared</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
@@ -1149,7 +1153,7 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>M3 — Scale above gate</t>
+          <t>M3 - Scale above gate</t>
         </is>
       </c>
       <c r="B8" s="18" t="n">
@@ -1208,7 +1212,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Q2 — Target</t>
+          <t>Q2 - Target</t>
         </is>
       </c>
       <c r="B9" s="18" t="n">
@@ -1264,6 +1268,7 @@
         <v/>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="25" t="inlineStr">
         <is>
@@ -1274,7 +1279,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>• ROAS (gate) uses first-year ARPPU — same basis as the task's ~100% anchor. Gate = 125%.</t>
+          <t>• ROAS (gate) uses first-year ARPPU - same basis as the task's ~100% anchor. Gate = 125%.</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1335,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Sensitivity — which metric moves ROAS most?</t>
+          <t>Sensitivity - which metric moves ROAS most?</t>
         </is>
       </c>
     </row>
@@ -1341,6 +1346,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
         <is>
@@ -1388,7 +1394,7 @@
       </c>
       <c r="E5" s="30" t="inlineStr">
         <is>
-          <t>UA-owned via CPP/PPO — high headroom</t>
+          <t>UA-owned via CPP/PPO - high headroom</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1418,7 @@
       </c>
       <c r="E6" s="30" t="inlineStr">
         <is>
-          <t>Product/paywall — most headroom, needs product</t>
+          <t>Product/paywall - most headroom, needs product</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1442,7 @@
       </c>
       <c r="E7" s="30" t="inlineStr">
         <is>
-          <t>Onboarding — shared with product</t>
+          <t>Onboarding - shared with product</t>
         </is>
       </c>
     </row>
@@ -1460,10 +1466,11 @@
       </c>
       <c r="E8" s="30" t="inlineStr">
         <is>
-          <t>UA-owned via structure/bids — fastest lever</t>
-        </is>
-      </c>
-    </row>
+          <t>UA-owned via structure/bids - fastest lever</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="25" t="inlineStr">
         <is>
@@ -1474,7 +1481,7 @@
     <row r="11">
       <c r="A11" s="32" t="inlineStr">
         <is>
-          <t>1) CPT efficiency (documented waste — fastest), 2) Trial→Paid (only 20%, most headroom), 3) tap→install CR via tool-CPPs/PPO.</t>
+          <t>1) CPT efficiency (documented waste - fastest), 2) Trial→Paid (only 20%, most headroom), 3) tap→install CR via tool-CPPs/PPO.</t>
         </is>
       </c>
     </row>
@@ -1518,6 +1525,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="33" t="inlineStr">
         <is>
@@ -1563,7 +1571,7 @@
       </c>
       <c r="E5" s="30" t="inlineStr">
         <is>
-          <t>Bid capped ~€3–5; brand is mostly cannibalised organic. Free budget.</t>
+          <t>Bid capped ~€3-5; brand is mostly cannibalised organic. Free budget.</t>
         </is>
       </c>
     </row>

</xml_diff>